<commit_message>
feat: add k6 load testing and fix E2E tests authentication issues
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium-report.xlsx
+++ b/selenium-tests/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
   <si>
     <t>SmartCanteen E2E Web Test Execution Report</t>
   </si>
@@ -31,10 +31,10 @@
     <t>DURATION (S)</t>
   </si>
   <si>
-    <t>100%</t>
-  </si>
-  <si>
-    <t>17.70</t>
+    <t>78%</t>
+  </si>
+  <si>
+    <t>87.31</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -109,6 +109,12 @@
     <t>Complete payment and generate digital canteen token pass</t>
   </si>
   <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>Active digital token pass not generated on dashboard</t>
+  </si>
+  <si>
     <t>TC-W007</t>
   </si>
   <si>
@@ -116,6 +122,9 @@
   </si>
   <si>
     <t>Claim order and pick up food</t>
+  </si>
+  <si>
+    <t>Claim Order button not visible on active pass card</t>
   </si>
   <si>
     <t>TC-W008</t>
@@ -137,7 +146,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -173,6 +182,17 @@
       <b/>
       <color rgb="15803D"/>
       <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="B91C1C"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="991B1B"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -292,7 +312,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -329,6 +349,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -712,10 +738,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="4">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>6</v>
@@ -758,7 +784,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="12">
-        <v>1024</v>
+        <v>1241</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>18</v>
@@ -778,7 +804,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="12">
-        <v>5032</v>
+        <v>3942</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>18</v>
@@ -798,7 +824,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="12">
-        <v>2596</v>
+        <v>2355</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>18</v>
@@ -818,7 +844,7 @@
         <v>17</v>
       </c>
       <c r="F11" s="12">
-        <v>1746</v>
+        <v>1631</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
@@ -838,7 +864,7 @@
         <v>17</v>
       </c>
       <c r="F12" s="12">
-        <v>145</v>
+        <v>2876</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>18</v>
@@ -854,51 +880,51 @@
       <c r="D13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>17</v>
+      <c r="E13" s="13" t="s">
+        <v>32</v>
       </c>
       <c r="F13" s="12">
-        <v>2139</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>18</v>
+        <v>2042</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>17</v>
-      </c>
       <c r="F14" s="12">
-        <v>1601</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>18</v>
+        <v>10010</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>33</v>
-      </c>
       <c r="D15" s="10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="12">
-        <v>1168</v>
+        <v>1098</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>18</v>
@@ -906,19 +932,19 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="12">
-        <v>988</v>
+        <v>951</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
feat: resolve all E2E Selenium suite test failures by implementing robust mock database query builder and routing fix
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium-report.xlsx
+++ b/selenium-tests/selenium-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t>SmartCanteen E2E Web Test Execution Report</t>
   </si>
@@ -31,10 +31,10 @@
     <t>DURATION (S)</t>
   </si>
   <si>
-    <t>78%</t>
-  </si>
-  <si>
-    <t>87.31</t>
+    <t>100%</t>
+  </si>
+  <si>
+    <t>20.20</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -109,12 +109,6 @@
     <t>Complete payment and generate digital canteen token pass</t>
   </si>
   <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>Active digital token pass not generated on dashboard</t>
-  </si>
-  <si>
     <t>TC-W007</t>
   </si>
   <si>
@@ -122,9 +116,6 @@
   </si>
   <si>
     <t>Claim order and pick up food</t>
-  </si>
-  <si>
-    <t>Claim Order button not visible on active pass card</t>
   </si>
   <si>
     <t>TC-W008</t>
@@ -146,7 +137,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -182,17 +173,6 @@
       <b/>
       <color rgb="15803D"/>
       <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="B91C1C"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="991B1B"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -312,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -349,12 +329,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -738,10 +712,10 @@
         <v>9</v>
       </c>
       <c r="C5" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>6</v>
@@ -784,7 +758,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="12">
-        <v>1241</v>
+        <v>856</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>18</v>
@@ -804,7 +778,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="12">
-        <v>3942</v>
+        <v>8166</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>18</v>
@@ -824,7 +798,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="12">
-        <v>2355</v>
+        <v>2883</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>18</v>
@@ -844,7 +818,7 @@
         <v>17</v>
       </c>
       <c r="F11" s="12">
-        <v>1631</v>
+        <v>1613</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
@@ -864,7 +838,7 @@
         <v>17</v>
       </c>
       <c r="F12" s="12">
-        <v>2876</v>
+        <v>52</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>18</v>
@@ -880,51 +854,51 @@
       <c r="D13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>32</v>
+      <c r="E13" s="11" t="s">
+        <v>17</v>
       </c>
       <c r="F13" s="12">
-        <v>2042</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>33</v>
+        <v>2059</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>32</v>
+      <c r="E14" s="11" t="s">
+        <v>17</v>
       </c>
       <c r="F14" s="12">
-        <v>10010</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>37</v>
+        <v>1534</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="12">
-        <v>1098</v>
+        <v>1068</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>18</v>
@@ -932,19 +906,19 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>17</v>
       </c>
       <c r="F16" s="12">
-        <v>951</v>
+        <v>912</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
chore: update selenium test reports
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium-report.xlsx
+++ b/selenium-tests/selenium-report.xlsx
@@ -34,7 +34,7 @@
     <t>100%</t>
   </si>
   <si>
-    <t>20.20</t>
+    <t>29.02</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -758,7 +758,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="12">
-        <v>856</v>
+        <v>9829</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>18</v>
@@ -778,7 +778,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="12">
-        <v>8166</v>
+        <v>7793</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>18</v>
@@ -798,7 +798,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="12">
-        <v>2883</v>
+        <v>3007</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>18</v>
@@ -818,7 +818,7 @@
         <v>17</v>
       </c>
       <c r="F11" s="12">
-        <v>1613</v>
+        <v>1629</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>18</v>
@@ -838,7 +838,7 @@
         <v>17</v>
       </c>
       <c r="F12" s="12">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>18</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="F13" s="12">
-        <v>2059</v>
+        <v>2067</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>18</v>
@@ -878,7 +878,7 @@
         <v>17</v>
       </c>
       <c r="F14" s="12">
-        <v>1534</v>
+        <v>1551</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>18</v>
@@ -898,7 +898,7 @@
         <v>17</v>
       </c>
       <c r="F15" s="12">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>18</v>
@@ -918,7 +918,7 @@
         <v>17</v>
       </c>
       <c r="F16" s="12">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>18</v>

</xml_diff>